<commit_message>
sinkronisasi pembaruan UI dan mobile token
</commit_message>
<xml_diff>
--- a/backend/public/templates/template_guru.xlsx
+++ b/backend/public/templates/template_guru.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -412,29 +412,40 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Siti Aminah</v>
+        <v>Rivia Guru</v>
       </c>
       <c r="B2" t="str">
-        <v>siti@example.com</v>
+        <v>riviadimong321@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>198001012010012001</v>
+        <v>198001012005011001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Ahmad Fauzi</v>
+        <v>Siti Aminah, S.Pd</v>
       </c>
       <c r="B3" t="str">
-        <v>ahmad@example.com</v>
+        <v>sitiaminah@guru.sekolah.sch.id</v>
       </c>
       <c r="C3" t="str">
-        <v>198102022011021002</v>
+        <v>198203152010012003</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Drs. Ahmad Fauzi, M.Pd</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ahmadfauzi@guru.sekolah.sch.id</v>
+      </c>
+      <c r="C4" t="str">
+        <v>197508222003121002</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>